<commit_message>
Assess ENG + cambio de modelo ENG + ajusto m_to_use + Actualizo predicciones.xlsx
</commit_message>
<xml_diff>
--- a/data/england/p6_deployment/data_preparation/df_emergency_fill.xlsx
+++ b/data/england/p6_deployment/data_preparation/df_emergency_fill.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O19"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,60 +441,65 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>mean_last_match_mean_rat_player_start_away_against</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>dif_mean_hei_player_start</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_int_rep_player_sub</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_rat_player_sub</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_val_player_start</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_age_player_sub</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_rat_player_start</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_age_player_start</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_pot_player_start</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_pot_player_sub</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_val_player_sub</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_int_rep_player_start</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_hei_player_sub</t>
         </is>
@@ -503,7 +508,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>AVat9lPF</t>
+          <t>z1q67ylB</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -520,11 +525,12 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Wplk7SgS</t>
+          <t>tvOWhxZH</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -541,11 +547,12 @@
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>tzSnG5Wr</t>
+          <t>U11vkTXq</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -562,321 +569,7 @@
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>beYTapn2</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>2TvL16Hk</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>AiyHLR8L</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>jkLFNmv9</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>2kGeEq1e</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>z1q67ylB</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>tvOWhxZH</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>U11vkTXq</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>INsZAAf3</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>SUdkBJln</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>x6HuiG3U</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>2Fanm72d</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>lpob9cJb</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>8QPOfb45</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>ERWFdKZh</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
DATA. Actualizo predicciones.xlsx con nuevos entrenamientos en SPA, ITA y GER.
</commit_message>
<xml_diff>
--- a/data/england/p6_deployment/data_preparation/df_emergency_fill.xlsx
+++ b/data/england/p6_deployment/data_preparation/df_emergency_fill.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>2ot8gOsJ</t>
+          <t>EqY7Orsg</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -511,9 +511,7 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
-      <c r="J2" t="n">
-        <v>-0.2251193662171381</v>
-      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
@@ -522,7 +520,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>SSZaQ4Ct</t>
+          <t>EcDtwrdn</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -535,9 +533,7 @@
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
-      <c r="J3" t="n">
-        <v>-0.2251193662171381</v>
-      </c>
+      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
@@ -546,7 +542,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>ShJjaSDs</t>
+          <t>EJlHkLuh</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -559,9 +555,7 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
-      <c r="J4" t="n">
-        <v>-0.2251193662171381</v>
-      </c>
+      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
@@ -570,7 +564,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>n9EQB5cm</t>
+          <t>zD1kyMQb</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -583,9 +577,7 @@
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
-      <c r="J5" t="n">
-        <v>-0.2251193662171381</v>
-      </c>
+      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
@@ -594,7 +586,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>tWiaepD6</t>
+          <t>rw5cZaeB</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -607,9 +599,7 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
-      <c r="J6" t="n">
-        <v>-0.2251193662171381</v>
-      </c>
+      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
@@ -618,7 +608,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>Y5lic6rf</t>
+          <t>zypxSHmo</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -631,9 +621,7 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
-      <c r="J7" t="n">
-        <v>-0.2251193662171381</v>
-      </c>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
@@ -642,7 +630,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>UiYgHRZP</t>
+          <t>ABRGMMB5</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -655,9 +643,7 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
-      <c r="J8" t="n">
-        <v>-0.2251193662171381</v>
-      </c>
+      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
@@ -666,7 +652,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>Gl6s8NdC</t>
+          <t>viJXIvBU</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -679,9 +665,7 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
-      <c r="J9" t="n">
-        <v>-0.2251193662171381</v>
-      </c>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
@@ -690,7 +674,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>OE9k61RO</t>
+          <t>rPPOK0tI</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -703,9 +687,7 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
-      <c r="J10" t="n">
-        <v>-0.2251193662171381</v>
-      </c>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
@@ -714,10 +696,12 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>fsjksfhd</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
+          <t>v5b6XwQN</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
@@ -734,10 +718,12 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>ltBAlx0M</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr"/>
+          <t>KMCY9qSa</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
@@ -754,10 +740,12 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>nywy5cp3</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr"/>
+          <t>2ot8gOsJ</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
@@ -771,6 +759,182 @@
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
     </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>SSZaQ4Ct</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>ShJjaSDs</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>UiYgHRZP</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>n9EQB5cm</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>Y5lic6rf</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>tWiaepD6</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>Gl6s8NdC</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>OE9k61RO</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizo predicciones.xlsx para el domingo y lunes por cuotas y missing
</commit_message>
<xml_diff>
--- a/data/england/p6_deployment/data_preparation/df_emergency_fill.xlsx
+++ b/data/england/p6_deployment/data_preparation/df_emergency_fill.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -493,7 +493,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>EqY7Orsg</t>
+          <t>KMCY9qSa</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -512,7 +512,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>EcDtwrdn</t>
+          <t>2ot8gOsJ</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -531,7 +531,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>EJlHkLuh</t>
+          <t>SSZaQ4Ct</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -547,329 +547,6 @@
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
     </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>zD1kyMQb</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>rw5cZaeB</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>zypxSHmo</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>ABRGMMB5</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>viJXIvBU</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>rPPOK0tI</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>v5b6XwQN</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>KMCY9qSa</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>2ot8gOsJ</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>SSZaQ4Ct</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>ShJjaSDs</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>UiYgHRZP</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>n9EQB5cm</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>Y5lic6rf</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>tWiaepD6</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>Gl6s8NdC</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>OE9k61RO</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>